<commit_message>
complete candidate identification architecture
</commit_message>
<xml_diff>
--- a/data/batch_results_10.xlsx
+++ b/data/batch_results_10.xlsx
@@ -426,17 +426,17 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="48" customWidth="1" min="19" max="19"/>
+    <col width="32" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,7 +574,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>A Greyhound, a Groundhog</t>
+          <t>A greyhound, a groundhog</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -584,14 +584,14 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Preschool</t>
+          <t>Early Elementary</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -600,20 +600,20 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>LOWER</t>
+          <t>ALIGNED</t>
         </is>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Picture Book</t>
+          <t>Children's Fiction</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Google Books</t>
+          <t>Open Library</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -670,14 +670,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Preschool</t>
+          <t>Early Elementary</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -686,11 +686,11 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LOWER</t>
+          <t>ALIGNED</t>
         </is>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -699,7 +699,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Google Books</t>
+          <t>Open Library</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -810,6 +810,11 @@
           <t>6th–8th Grade</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>11–14</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Fiction</t>
@@ -825,14 +830,53 @@
           <t>6th–8th Grade Fiction List (user-provided)</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>A Wrinkle in Time</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Madeleine L'Engle</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Elementary</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" t="n">
+        <v>10</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>LOWER</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>LOWER</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Science Fiction</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Google Books</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>The request to Open Library timed out.</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -852,6 +896,11 @@
           <t>9th–10th Grade</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>14–16</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Not specified</t>
@@ -867,14 +916,53 @@
           <t>9C / 9R / 10C / 10R Summer Reading 2026</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pemmican Wars</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Katherena Vermette</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Middle School</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>LOWER</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>3</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Graphic Novel</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Google Books</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Could not find book: A Girl Called Echo Vol. 1</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -894,6 +982,11 @@
           <t>9th–10th Grade</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14–16</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>Not specified</t>
@@ -909,14 +1002,53 @@
           <t>9C / 9R / 10C / 10R Summer Reading 2026</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>16 Forever</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Lance Rubin</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>High School</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>14</v>
+      </c>
+      <c r="L7" t="n">
+        <v>18</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>ALIGNED</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Young Adult Fiction</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Google Books</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Could not find book: 16 Forever</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>
@@ -958,7 +1090,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Could not find book: A Scatter of Light</t>
+          <t>No candidate books were found.</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1166,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Historical Nonfiction</t>
+          <t>Historical Non-Fiction</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Google Books</t>
+          <t>Open Library</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1086,7 +1218,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Devil's Plaything</t>
+          <t>A Deadly Wandering</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1096,18 +1228,18 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Adult</t>
+          <t>High School</t>
         </is>
       </c>
       <c r="K10" t="n">
+        <v>14</v>
+      </c>
+      <c r="L10" t="n">
         <v>18</v>
       </c>
-      <c r="L10" t="n">
-        <v>99</v>
-      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>HIGHER</t>
+          <t>ALIGNED</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1120,7 +1252,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Thriller</t>
+          <t>Non-Fiction</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1202,7 +1334,7 @@
         </is>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>

</xml_diff>